<commit_message>
Keep Excel invoice sections intact across pages
</commit_message>
<xml_diff>
--- a/site/form/samples/form-rows-modern.xlsx
+++ b/site/form/samples/form-rows-modern.xlsx
@@ -10,7 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="請求書" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'請求書'!$1:$15</definedName>
+    <definedName name="_bdf.Print_TitleScope" localSheetId="0">'請求書'!$A$15:$H$16</definedName>
+    <definedName name="_bdf.Print_KeepTogether" localSheetId="0">'請求書'!$F$18:$H$20,'請求書'!$A$22:$H$25,'請求書'!$A$27:$H$31</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'請求書'!$15:$15</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'請求書'!$A$1:$H$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Keep Excel invoice sections intact across pages (#93)
</commit_message>
<xml_diff>
--- a/site/form/samples/form-rows-modern.xlsx
+++ b/site/form/samples/form-rows-modern.xlsx
@@ -10,7 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="請求書" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'請求書'!$1:$15</definedName>
+    <definedName name="_bdf.Print_TitleScope" localSheetId="0">'請求書'!$A$15:$H$16</definedName>
+    <definedName name="_bdf.Print_KeepTogether" localSheetId="0">'請求書'!$F$18:$H$20,'請求書'!$A$22:$H$25,'請求書'!$A$27:$H$31</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'請求書'!$15:$15</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'請求書'!$A$1:$H$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>